<commit_message>
docs: REQUIREMENTS.xlsx statuses for completed rows
</commit_message>
<xml_diff>
--- a/docs/qa-handover/requirements/REQUIREMENTS.xlsx
+++ b/docs/qa-handover/requirements/REQUIREMENTS.xlsx
@@ -1859,12 +1859,12 @@
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>All 13 companies NULL statutory ids (SCHEMA_AUDIT S-24); no UI</t>
+          <t>All 13 companies NULL statutory ids (SCHEMA_AUDIT S-24); no UI | fix 0c02438: org masters CRUD with company statutory ID validation (Admin → Org masters)</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -1979,12 +1979,12 @@
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>core.employee_family and core.profile_change_requests unreferenced in code (SCHEMA_AUDIT S-23)</t>
+          <t>core.employee_family and core.profile_change_requests unreferenced in code (SCHEMA_AUDIT S-23) | fix 0c02438: ESS family/nominee change → family_update chain → HR apply</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -2327,12 +2327,12 @@
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>company-scope.ts requireRunInScope; B-16 open in QA REPORT; fix in progress (uncommitted separation.router.ts)</t>
+          <t>company-scope.ts requireRunInScope; B-16 open in QA REPORT; fix in progress (uncommitted separation.router.ts) | fix 82e1608: entity-scoped grants require org unit (API+UI); tests access-control</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
@@ -2786,12 +2786,12 @@
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>frontend/src/app/nav-config.ts; QA beta crawl 57 routes</t>
+          <t>frontend/src/app/nav-config.ts; QA beta crawl 57 routes | fix 48bb121: route guard (route-guard.ts) + 403 state; unit tests</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr"/>
@@ -3340,12 +3340,12 @@
       </c>
       <c r="I50" s="4" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>No evidence (plans/launch-readiness/03-PHASE-STATUS.md Phase 0 open)</t>
+          <t>No evidence (plans/launch-readiness/03-PHASE-STATUS.md Phase 0 open) | fix 5bb73be: scripts/backup.sh + restore.sh, drill evidence fix-verify/backup/EVIDENCE.md; WAL/PITR still infra</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr"/>
@@ -3621,7 +3621,7 @@
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>kent-connector.ts/kent-sync.job.ts: fail-closed guard (pack31); real Kent adapter/protocol not available (sponsor to supply)</t>
+          <t>kent-connector.ts/kent-sync.job.ts: fail-closed guard (pack31); real Kent adapter/protocol not available (sponsor to supply) | fix a89640f: KentHttpConnector + simulator + docs/integrations/KENT.md; pending real Kent credentials</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
@@ -8621,12 +8621,12 @@
       </c>
       <c r="I142" s="4" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>declareInvestment/verifyDeclaration require payroll.run.manage (statutory.router.ts) - no employee self-service</t>
+          <t>declareInvestment/verifyDeclaration require payroll.run.manage (statutory.router.ts) - no employee self-service | fix c017496: /my/tax declarations + proofs + regime; windows in settings</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr">
@@ -8680,12 +8680,12 @@
       </c>
       <c r="I143" s="4" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>generateForm24QSummary function only (tds.ts:363) with no route; no Form 16 route; Alumni page references Form 16 without backend</t>
+          <t>generateForm24QSummary function only (tds.ts:363) with no route; no Form 16 route; Alumni page references Form 16 without backend | fix c017496: Form 24Q CSV per quarter, Form 16 PDF (payroll + ESS/alumni)</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
@@ -8738,12 +8738,12 @@
       </c>
       <c r="I144" s="4" t="inlineStr">
         <is>
-          <t>Missing</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>pay.tds_challans unreferenced (SCHEMA_AUDIT S-23)</t>
+          <t>pay.tds_challans unreferenced (SCHEMA_AUDIT S-23) | fix c017496: TDS challans + monthly reconciliation (Payroll → TDS compliance)</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -10813,12 +10813,12 @@
       </c>
       <c r="I180" s="3" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J180" s="2" t="inlineStr">
         <is>
-          <t>/lifecycle/separations/apply; B-04 IDOR fix in progress (separation.router.ts uncommitted)</t>
+          <t>/lifecycle/separations/apply; B-04 IDOR fix in progress (separation.router.ts uncommitted) | fix f09dbc6: ESS resignation for signed-in employee, notice from policy</t>
         </is>
       </c>
       <c r="K180" s="2" t="inlineStr">

</xml_diff>

<commit_message>
reqs: joining form RML/HR/02/01 field map + Enterprise Blueprint gap; 55 new REQUIREMENTS rows (RQ-JF-001..022, RQ-BP-*), xlsx + summary updated
</commit_message>
<xml_diff>
--- a/docs/qa-handover/requirements/REQUIREMENTS.xlsx
+++ b/docs/qa-handover/requirements/REQUIREMENTS.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Requirements'!$A$1:$K$259</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Requirements'!$A$1:$K$314</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$1:$F$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K259"/>
+  <dimension ref="A1:K314"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -15287,8 +15287,3249 @@
       </c>
       <c r="K259" s="2" t="inlineStr"/>
     </row>
+    <row r="260">
+      <c r="A260" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-001</t>
+        </is>
+      </c>
+      <c r="B260" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C260" s="2" t="inlineStr">
+        <is>
+          <t>Pre-join → employee conversion applies the same validation as HR create/import: PAN AAAAA9999A, Aadhaar 12 digits + Verhoeff, UAN 12 digits, IFSC AAAA0XXXXXX, account 9–18 digits, 18+ on DOJ, duplicate PAN/Aadhaar/UAN/ESIC/bank account across employees.</t>
+        </is>
+      </c>
+      <c r="D260" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E260" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F260" s="2" t="inlineStr">
+        <is>
+          <t>hr_ops, candidate</t>
+        </is>
+      </c>
+      <c r="G260" s="2" t="inlineStr">
+        <is>
+          <t>1. Create a candidate and open the pre-join link
+2. Submit Aadhaar 234567890123 (bad checksum), IFSC ABCD1234567, account 1234567A
+3. Expect field errors on the portal
+4. Force-submit via API and try Convert as hr_ops
+5. Expect 400 with the same messages POST /employees gives; no employee created</t>
+        </is>
+      </c>
+      <c r="H260" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I260" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J260" s="2" t="inlineStr">
+        <is>
+          <t>lifecycle/onboarding/prejoin-schema.ts checks lengths only; onboarding.service.ts convert inserts core.employees directly; duplicate check = email/mobile/PAN only. Importer rules in bulk/importers/employees.ts.</t>
+        </is>
+      </c>
+      <c r="K260" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-002</t>
+        </is>
+      </c>
+      <c r="B261" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C261" s="2" t="inlineStr">
+        <is>
+          <t>Personal extension captured on joining and editable by HR: father's name, spouse name, marriage date, nationality, country of origin, religion, caste (optional, restricted), height, weight, physically disabled (Y/N + %), identification mark, passport no. + validity, driving licence no., name as per Aadhaar.</t>
+        </is>
+      </c>
+      <c r="D261" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E261" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F261" s="2" t="inlineStr">
+        <is>
+          <t>candidate, hr_ops, employee (view own)</t>
+        </is>
+      </c>
+      <c r="G261" s="2" t="inlineStr">
+        <is>
+          <t>1. Pre-join portal shows every field in §2 of the form
+2. HR People &gt; Edit shows and saves them
+3. Profile &gt; Personal shows them; caste/religion visible only to HR roles</t>
+        </is>
+      </c>
+      <c r="H261" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I261" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J261" s="2" t="inlineStr">
+        <is>
+          <t>No columns on core.employees (JOINING_FORM_MAP rows 13–31).</t>
+        </is>
+      </c>
+      <c r="K261" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-003</t>
+        </is>
+      </c>
+      <c r="B262" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C262" s="2" t="inlineStr">
+        <is>
+          <t>Gender options Male / Female / Transgender, collected on the pre-join portal and copied on conversion.</t>
+        </is>
+      </c>
+      <c r="D262" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E262" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F262" s="2" t="inlineStr">
+        <is>
+          <t>candidate, hr_ops</t>
+        </is>
+      </c>
+      <c r="G262" s="2" t="inlineStr">
+        <is>
+          <t>1. Submit pre-join with gender Transgender
+2. Convert
+3. Profile shows Transgender; ESIC/PF exports carry it</t>
+        </is>
+      </c>
+      <c r="H262" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I262" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J262" s="2" t="inlineStr">
+        <is>
+          <t>employee-master.router.ts enum Male/Female/Other; prejoin has no gender; convert leaves gender NULL.</t>
+        </is>
+      </c>
+      <c r="K262" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-004</t>
+        </is>
+      </c>
+      <c r="B263" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C263" s="2" t="inlineStr">
+        <is>
+          <t>Marital status options Single / Married / Widow / Widower / Divorcee (EPF Form 11), captured on pre-join and HR create/edit.</t>
+        </is>
+      </c>
+      <c r="D263" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E263" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F263" s="2" t="inlineStr">
+        <is>
+          <t>candidate, hr_ops</t>
+        </is>
+      </c>
+      <c r="G263" s="2" t="inlineStr">
+        <is>
+          <t>1. HR edit employee &gt; marital status Widow &gt; Save
+2. Profile shows Widow; audit row written</t>
+        </is>
+      </c>
+      <c r="H263" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I263" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J263" s="2" t="inlineStr">
+        <is>
+          <t>core.employees.marital_status exists (display only); not in POST/PATCH /employees or prejoin.</t>
+        </is>
+      </c>
+      <c r="K263" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-005</t>
+        </is>
+      </c>
+      <c r="B264" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C264" s="2" t="inlineStr">
+        <is>
+          <t>HR create/edit (POST/PATCH /employees, importer columns, EmployeeFormDrawer) covers every master field: personal e-mail, marital status, blood group, both addresses, emergency contact, plant, cost centre, functional manager.</t>
+        </is>
+      </c>
+      <c r="D264" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E264" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F264" s="2" t="inlineStr">
+        <is>
+          <t>hr_ops, hr_head</t>
+        </is>
+      </c>
+      <c r="G264" s="2" t="inlineStr">
+        <is>
+          <t>1. HR keys a paper joining form for a walk-in joiner via People &gt; New
+2. All §1–§5 and §9 fields save
+3. Download importer template: same columns present</t>
+        </is>
+      </c>
+      <c r="H264" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I264" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J264" s="2" t="inlineStr">
+        <is>
+          <t>employee-master.router.ts fields omit personal_email, marital_status, blood_group, addresses, emergency, plant, cost centre.</t>
+        </is>
+      </c>
+      <c r="K264" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-006</t>
+        </is>
+      </c>
+      <c r="B265" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C265" s="2" t="inlineStr">
+        <is>
+          <t>Structured present and permanent address: house/flat, locality, city/village, post office, police station/thana, district, state (code), country, PIN (6 digits); "same as present" option; state drives PT/LWF.</t>
+        </is>
+      </c>
+      <c r="D265" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E265" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F265" s="2" t="inlineStr">
+        <is>
+          <t>candidate, hr_ops</t>
+        </is>
+      </c>
+      <c r="G265" s="2" t="inlineStr">
+        <is>
+          <t>1. Enter PIN 7000 → error "PIN must be 6 digits"
+2. Tick same as present → permanent copies
+3. Profile shows formatted address; PT state = address/work-location rule per policy</t>
+        </is>
+      </c>
+      <c r="H265" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I265" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J265" s="2" t="inlineStr">
+        <is>
+          <t>present_address/permanent_address are single text columns (prejoin min 5 chars).</t>
+        </is>
+      </c>
+      <c r="K265" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-007</t>
+        </is>
+      </c>
+      <c r="B266" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C266" s="2" t="inlineStr">
+        <is>
+          <t>Emergency contact: name, relationship (persisted), mobile (10 digits), alternate number, address; at least one required.</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E266" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F266" s="2" t="inlineStr">
+        <is>
+          <t>candidate, employee, hr_ops</t>
+        </is>
+      </c>
+      <c r="G266" s="2" t="inlineStr">
+        <is>
+          <t>1. Submit pre-join with relationship "Brother"
+2. Convert
+3. Profile shows relationship Brother</t>
+        </is>
+      </c>
+      <c r="H266" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I266" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J266" s="2" t="inlineStr">
+        <is>
+          <t>emergencyContactRelation is collected by the prejoin portal and dropped on conversion (no column); no alternate/address.</t>
+        </is>
+      </c>
+      <c r="K266" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-008</t>
+        </is>
+      </c>
+      <c r="B267" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C267" s="2" t="inlineStr">
+        <is>
+          <t>Bank details: bank, branch, account holder name, account no., IFSC, account type (savings/current); warn when holder name differs from employee name.</t>
+        </is>
+      </c>
+      <c r="D267" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E267" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F267" s="2" t="inlineStr">
+        <is>
+          <t>candidate, hr_ops, payroll_admin</t>
+        </is>
+      </c>
+      <c r="G267" s="2" t="inlineStr">
+        <is>
+          <t>1. Enter holder name differing from employee name
+2. Expect amber warning, HR must confirm
+3. Bank file uses holder name</t>
+        </is>
+      </c>
+      <c r="H267" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I267" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J267" s="2" t="inlineStr">
+        <is>
+          <t>No branch/holder/type columns; prejoin label hard-codes "Savings".</t>
+        </is>
+      </c>
+      <c r="K267" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-009</t>
+        </is>
+      </c>
+      <c r="B268" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C268" s="2" t="inlineStr">
+        <is>
+          <t>Education grid (qualification, institute/university, year of passing, specialization, % / CGPA), multiple rows, on pre-join, HR edit and profile.</t>
+        </is>
+      </c>
+      <c r="D268" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E268" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F268" s="2" t="inlineStr">
+        <is>
+          <t>candidate, hr_ops, employee</t>
+        </is>
+      </c>
+      <c r="G268" s="2" t="inlineStr">
+        <is>
+          <t>1. Add 2 rows on pre-join
+2. After conversion, Profile &gt; Education shows both
+3. HR can edit; audit written</t>
+        </is>
+      </c>
+      <c r="H268" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I268" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J268" s="2" t="inlineStr">
+        <is>
+          <t>No table/API/UI.</t>
+        </is>
+      </c>
+      <c r="K268" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-010</t>
+        </is>
+      </c>
+      <c r="B269" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C269" s="2" t="inlineStr">
+        <is>
+          <t>Certification grid (name, issuing organisation, date, specialization, grade/score, expiry date) with expiry alerts.</t>
+        </is>
+      </c>
+      <c r="D269" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E269" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F269" s="2" t="inlineStr">
+        <is>
+          <t>candidate, hr_ops</t>
+        </is>
+      </c>
+      <c r="G269" s="2" t="inlineStr">
+        <is>
+          <t>1. Add a certificate expiring in 20 days
+2. Expect it in HR expiry alerts</t>
+        </is>
+      </c>
+      <c r="H269" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I269" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J269" s="2" t="inlineStr">
+        <is>
+          <t>No table.</t>
+        </is>
+      </c>
+      <c r="K269" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-011</t>
+        </is>
+      </c>
+      <c r="B270" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C270" s="2" t="inlineStr">
+        <is>
+          <t>Previous employment grid (employer, designation, from, to, reason for leaving; optional last CTC, previous PF/UAN).</t>
+        </is>
+      </c>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E270" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F270" s="2" t="inlineStr">
+        <is>
+          <t>candidate, hr_ops</t>
+        </is>
+      </c>
+      <c r="G270" s="2" t="inlineStr">
+        <is>
+          <t>1. Add 2 employers on pre-join
+2. Profile &gt; Experience lists them; total experience computed</t>
+        </is>
+      </c>
+      <c r="H270" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I270" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J270" s="2" t="inlineStr">
+        <is>
+          <t>Only onboarding_candidates.previous_company (single, not copied). See RQ-CORE-024.</t>
+        </is>
+      </c>
+      <c r="K270" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-012</t>
+        </is>
+      </c>
+      <c r="B271" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C271" s="2" t="inlineStr">
+        <is>
+          <t>Family grid captured on pre-join: name, relation, gender, DOB/age, Aadhaar, pre-existing disease (restricted), residing with employee (Y/N, else town/state), ESIC dependent flag.</t>
+        </is>
+      </c>
+      <c r="D271" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E271" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F271" s="2" t="inlineStr">
+        <is>
+          <t>candidate, employee, hr_ops</t>
+        </is>
+      </c>
+      <c r="G271" s="2" t="inlineStr">
+        <is>
+          <t>1. Add spouse and child on pre-join
+2. After conversion Family tab lists both
+3. Disease visible to HR-medical only</t>
+        </is>
+      </c>
+      <c r="H271" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I271" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J271" s="2" t="inlineStr">
+        <is>
+          <t>core.employee_family has name/relation/dob/aadhaar/esic/nominee; no gender, disease, residing; not in prejoin.</t>
+        </is>
+      </c>
+      <c r="K271" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-013</t>
+        </is>
+      </c>
+      <c r="B272" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C272" s="2" t="inlineStr">
+        <is>
+          <t>Scheme-wise nominations: PF (Form 2), EPS, gratuity (Form F), ESIC (s.71), group insurance. Each holds nominee, relationship, address, age, share % (100 per scheme), minor guardian, and Form F witnesses + employer certification; a new nomination supersedes the previous one.</t>
+        </is>
+      </c>
+      <c r="D272" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E272" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F272" s="2" t="inlineStr">
+        <is>
+          <t>employee, hr_ops</t>
+        </is>
+      </c>
+      <c r="G272" s="2" t="inlineStr">
+        <is>
+          <t>1. Employee nominates spouse 100% for gratuity and mother 100% for PF
+2. Both saved separately; shares checked per scheme
+3. Form F PDF lists spouse only</t>
+        </is>
+      </c>
+      <c r="H272" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I272" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J272" s="2" t="inlineStr">
+        <is>
+          <t>Single is_nominee + nominee_share_pct on employee_family for all schemes (family.service.ts).</t>
+        </is>
+      </c>
+      <c r="K272" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-014</t>
+        </is>
+      </c>
+      <c r="B273" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C273" s="2" t="inlineStr">
+        <is>
+          <t>EPF Form 11 history captured: earlier EPF member, earlier EPS member, member before 01-Sep-2014, previous UAN/PF no., exit date, scheme certificate, PPO, EPF/EPS withdrawn, international worker + country + passport; PF engine uses it for EPS eligibility (no EPS for post-Sep-2014 new members with PF wages &gt; ₹15,000; international workers uncapped).</t>
+        </is>
+      </c>
+      <c r="D273" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E273" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F273" s="2" t="inlineStr">
+        <is>
+          <t>candidate, hr_ops, payroll_admin</t>
+        </is>
+      </c>
+      <c r="G273" s="2" t="inlineStr">
+        <is>
+          <t>1. Joiner: first-time member, basic ₹25,000
+2. Run payroll: employer 12% goes fully to EPF, EPS 0
+3. Joiner with pre-2014 membership: EPS 8.33% of ₹15,000</t>
+        </is>
+      </c>
+      <c r="H273" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I273" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J273" s="2" t="inlineStr">
+        <is>
+          <t>No fields; statutory/pf.ts cannot decide EPS eligibility per member.</t>
+        </is>
+      </c>
+      <c r="K273" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-015</t>
+        </is>
+      </c>
+      <c r="B274" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C274" s="2" t="inlineStr">
+        <is>
+          <t>ESIC Form-1 data: dispensary, branch office, previous insurance no., previous employer code, family residing details; export for IP registration.</t>
+        </is>
+      </c>
+      <c r="D274" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E274" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F274" s="2" t="inlineStr">
+        <is>
+          <t>hr_ops</t>
+        </is>
+      </c>
+      <c r="G274" s="2" t="inlineStr">
+        <is>
+          <t>1. ESIC-eligible joiner: HR completes ESIC block
+2. Export "ESIC new IP" sheet with all Form-1 fields</t>
+        </is>
+      </c>
+      <c r="H274" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I274" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J274" s="2" t="inlineStr">
+        <is>
+          <t>None; ESIC registration is a portal task (RQ-SVC-002) but HRMS must hold the data.</t>
+        </is>
+      </c>
+      <c r="K274" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-016</t>
+        </is>
+      </c>
+      <c r="B275" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C275" s="2" t="inlineStr">
+        <is>
+          <t>Declaration and consent are recorded: §10 joining declaration, EPF undertaking (Aadhaar eKYC + fund transfer), ESIC declaration, DPDP consent for health data. Each record keeps the text version, timestamp, IP and an e-signature or uploaded signature.</t>
+        </is>
+      </c>
+      <c r="D275" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E275" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F275" s="2" t="inlineStr">
+        <is>
+          <t>candidate, hr_ops</t>
+        </is>
+      </c>
+      <c r="G275" s="2" t="inlineStr">
+        <is>
+          <t>1. Pre-join submit is disabled until the declaration is ticked and signed
+2. HR sees "Declared 19-Oct-2026 10:02 IST from IP …"</t>
+        </is>
+      </c>
+      <c r="H275" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I275" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J275" s="2" t="inlineStr">
+        <is>
+          <t>Prejoin submit has no declaration/consent; prv.consents not wired.</t>
+        </is>
+      </c>
+      <c r="K275" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-017</t>
+        </is>
+      </c>
+      <c r="B276" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C276" s="2" t="inlineStr">
+        <is>
+          <t>Document checklist with upload and verification: photo, PAN, Aadhaar, bank proof, education, experience/relieving, last payslips, passport/DL, medical fitness, disability certificate. Mandatory items per category; HR verifies or rejects each with a reason; files go to the employee repository.</t>
+        </is>
+      </c>
+      <c r="D276" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E276" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F276" s="2" t="inlineStr">
+        <is>
+          <t>candidate, hr_ops, employee</t>
+        </is>
+      </c>
+      <c r="G276" s="2" t="inlineStr">
+        <is>
+          <t>1. Pre-join: upload PAN, Aadhaar, cheque, photo
+2. HR review shows each with Verify/Reject
+3. Convert blocked while a mandatory doc is missing or rejected
+4. Profile &gt; Documents lists them</t>
+        </is>
+      </c>
+      <c r="H276" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I276" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J276" s="2" t="inlineStr">
+        <is>
+          <t>core.documents + doc.types (pan, aadhaar, appointment, medical_fitness) but no upload/verify API or UI; photo_path never set.</t>
+        </is>
+      </c>
+      <c r="K276" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-018</t>
+        </is>
+      </c>
+      <c r="B277" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C277" s="2" t="inlineStr">
+        <is>
+          <t>Medical questionnaire (self and family history, medications, limitations, surgeries, allergies, height/weight/BMI, lifestyle, emergency medical needs, sports) is stored in a restricted store with DPDP consent and its own permission; managers never see it.</t>
+        </is>
+      </c>
+      <c r="D277" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E277" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F277" s="2" t="inlineStr">
+        <is>
+          <t>candidate, hr (medical)</t>
+        </is>
+      </c>
+      <c r="G277" s="2" t="inlineStr">
+        <is>
+          <t>1. Candidate completes medical section
+2. Manager opening Profile sees no medical tab
+3. HR-medical role sees it; access is audited</t>
+        </is>
+      </c>
+      <c r="H277" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I277" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J277" s="2" t="inlineStr">
+        <is>
+          <t>None (variants B and C pages 5–6 / 9–10).</t>
+        </is>
+      </c>
+      <c r="K277" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-019</t>
+        </is>
+      </c>
+      <c r="B278" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C278" s="2" t="inlineStr">
+        <is>
+          <t>HR office-use checklist on the joining record: joining formalities complete, master created, payroll set up (salary assigned), ID card/access, BGV initiated (Y/N/NA), induction scheduled (date), HR representative sign-off with date.</t>
+        </is>
+      </c>
+      <c r="D278" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E278" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F278" s="2" t="inlineStr">
+        <is>
+          <t>hr_ops</t>
+        </is>
+      </c>
+      <c r="G278" s="2" t="inlineStr">
+        <is>
+          <t>1. Convert a joiner
+2. Checklist shows 7 items; payroll item done only when a salary is assigned
+3. HR signs off; timestamp shown</t>
+        </is>
+      </c>
+      <c r="H278" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I278" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J278" s="2" t="inlineStr">
+        <is>
+          <t>Tasks it_email/it_laptop/it_biometric/admin_id_card/hr_induction only (task-fanout.service.ts); no BGV/payroll task or sign-off.</t>
+        </is>
+      </c>
+      <c r="K278" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-020</t>
+        </is>
+      </c>
+      <c r="B279" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C279" s="2" t="inlineStr">
+        <is>
+          <t>Pre-filled PDF output from the master: Employee Joining Form RML/HR/02/01, Form F, ESIC Form-1 data, EPF Form 11, ready for e-sign or wet signature and stored in documents.</t>
+        </is>
+      </c>
+      <c r="D279" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E279" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F279" s="2" t="inlineStr">
+        <is>
+          <t>hr_ops</t>
+        </is>
+      </c>
+      <c r="G279" s="2" t="inlineStr">
+        <is>
+          <t>1. Profile &gt; Documents &gt; Generate joining pack
+2. PDF matches the RML layout with data filled</t>
+        </is>
+      </c>
+      <c r="H279" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I279" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J279" s="2" t="inlineStr">
+        <is>
+          <t>Letters engine has no such templates.</t>
+        </is>
+      </c>
+      <c r="K279" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-021</t>
+        </is>
+      </c>
+      <c r="B280" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C280" s="2" t="inlineStr">
+        <is>
+          <t>Employment type maps the form's Permanent / Contract / Trainee / Consultant (+ Apprentice, Intern, Fixed-term) onto one documented field; conversion does not hard-code probationary.</t>
+        </is>
+      </c>
+      <c r="D280" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E280" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F280" s="2" t="inlineStr">
+        <is>
+          <t>hr_ops</t>
+        </is>
+      </c>
+      <c r="G280" s="2" t="inlineStr">
+        <is>
+          <t>1. Convert a consultant
+2. Employee shows type Consultant, not probationary</t>
+        </is>
+      </c>
+      <c r="H280" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I280" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J280" s="2" t="inlineStr">
+        <is>
+          <t>category + contract_type enums overlap; convert sets contract_type=probationary.</t>
+        </is>
+      </c>
+      <c r="K280" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="2" t="inlineStr">
+        <is>
+          <t>RQ-JF-022</t>
+        </is>
+      </c>
+      <c r="B281" s="2" t="inlineStr">
+        <is>
+          <t>JF Joining form RML/HR/02/01</t>
+        </is>
+      </c>
+      <c r="C281" s="2" t="inlineStr">
+        <is>
+          <t>Multi-step joining form UI (pre-join portal and HR "New joiner") in the RML/HR/02/01 section order with repeating-row editors, save draft, progress, review page, mobile one-hand layout (360–430px), WCAG AA.</t>
+        </is>
+      </c>
+      <c r="D281" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs RML/HR/02/01 Employee Joining Form (3 variants, 04 Sep 2026); /workspace/STATE/JOINING_FORM_MAP.md</t>
+        </is>
+      </c>
+      <c r="E281" s="2" t="inlineStr">
+        <is>
+          <t>CORE-01 / LC-01</t>
+        </is>
+      </c>
+      <c r="F281" s="2" t="inlineStr">
+        <is>
+          <t>candidate, hr_ops</t>
+        </is>
+      </c>
+      <c r="G281" s="2" t="inlineStr">
+        <is>
+          <t>1. On a 390px phone complete all steps
+2. Draft survives reload
+3. axe reports 0 serious issues</t>
+        </is>
+      </c>
+      <c r="H281" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I281" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J281" s="2" t="inlineStr">
+        <is>
+          <t>PrejoinPortalPage.tsx is a single page with 12 fields.</t>
+        </is>
+      </c>
+      <c r="K281" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-002</t>
+        </is>
+      </c>
+      <c r="B282" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C282" s="2" t="inlineStr">
+        <is>
+          <t>Position kept separate from designation; each position holds sanctioned HC, occupied HC, vacancy</t>
+        </is>
+      </c>
+      <c r="D282" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §1/§6</t>
+        </is>
+      </c>
+      <c r="E282" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §1/§6</t>
+        </is>
+      </c>
+      <c r="F282" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G282" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Position kept separate from designation; each position holds sanctioned HC, occupied HC, vacancy
+3. Expect the behaviour in blueprint §1/§6; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H282" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I282" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J282" s="2" t="inlineStr">
+        <is>
+          <t>No position table or API.</t>
+        </is>
+      </c>
+      <c r="K282" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-020</t>
+        </is>
+      </c>
+      <c r="B283" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C283" s="2" t="inlineStr">
+        <is>
+          <t>All major HR transactions effective-dated, preserving old values (transfer, promotion, revision, designation/grade, dept/location, RM, employment-type change)</t>
+        </is>
+      </c>
+      <c r="D283" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §4; widens RQ-LC-011</t>
+        </is>
+      </c>
+      <c r="E283" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §4</t>
+        </is>
+      </c>
+      <c r="F283" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G283" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: All major HR transactions effective-dated, preserving old values (transfer, promotion, revision, designation/grade, dept
+3. Expect the behaviour in blueprint §4; go-live: Core</t>
+        </is>
+      </c>
+      <c r="H283" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I283" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J283" s="2" t="inlineStr">
+        <is>
+          <t>Transfers + salary revisions effective-dated; designation/grade/RM/type edits via PATCH are immediate (no effective date, no history row).</t>
+        </is>
+      </c>
+      <c r="K283" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-040</t>
+        </is>
+      </c>
+      <c r="B284" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C284" s="2" t="inlineStr">
+        <is>
+          <t>Position master (position ID/name, entity, division, location, establishment, dept, section, designation, grade, job family, job level, cost centre, budgeted/sanctioned/occupied HC, vacancy, reporting position)</t>
+        </is>
+      </c>
+      <c r="D284" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §6</t>
+        </is>
+      </c>
+      <c r="E284" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §6</t>
+        </is>
+      </c>
+      <c r="F284" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G284" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Position master (position ID/name, entity, division, location, establishment, dept, section, designation, grade, job fam
+3. Expect the behaviour in blueprint §6; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H284" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I284" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J284" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="K284" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-080</t>
+        </is>
+      </c>
+      <c r="B285" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C285" s="2" t="inlineStr">
+        <is>
+          <t>OT types: normal, holiday, weekly-off, night OT, shift allowance, comp-off</t>
+        </is>
+      </c>
+      <c r="D285" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §11; widens RQ-ATT-019, RQ-PAY-022</t>
+        </is>
+      </c>
+      <c r="E285" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §11</t>
+        </is>
+      </c>
+      <c r="F285" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G285" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: OT types: normal, holiday, weekly-off, night OT, shift allowance, comp-off
+3. Expect the behaviour in blueprint §11; go-live: Core</t>
+        </is>
+      </c>
+      <c r="H285" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I285" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J285" s="2" t="inlineStr">
+        <is>
+          <t>att.overtime_entries has one type; comp-off credit for WO; no per-type OT rates.</t>
+        </is>
+      </c>
+      <c r="K285" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-110</t>
+        </is>
+      </c>
+      <c r="B286" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C286" s="2" t="inlineStr">
+        <is>
+          <t>Pre-payroll validation: missing bank/PAN/UAN/ESIC, abnormal salary change, negative salary, excess OT, duplicate employees, bank changes, major variances</t>
+        </is>
+      </c>
+      <c r="D286" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §14; widens RQ-PAY-008</t>
+        </is>
+      </c>
+      <c r="E286" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §14</t>
+        </is>
+      </c>
+      <c r="F286" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G286" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Pre-payroll validation: missing bank/PAN/UAN/ESIC, abnormal salary change, negative salary, excess OT, duplicate employe
+3. Expect the behaviour in blueprint §14; go-live: Core</t>
+        </is>
+      </c>
+      <c r="H286" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I286" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J286" s="2" t="inlineStr">
+        <is>
+          <t>variance.service.ts (negative net, variance anomalies); bank-file refuses missing bank/IFSC at output time only; no pre-run missing-PAN/UAN/ESIC, excess-OT or bank-change alert.</t>
+        </is>
+      </c>
+      <c r="K286" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-111</t>
+        </is>
+      </c>
+      <c r="B287" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C287" s="2" t="inlineStr">
+        <is>
+          <t>Excel import engine: template → upload → validate → error report → preview → maker → checker → approve → import → transaction ID → audit</t>
+        </is>
+      </c>
+      <c r="D287" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §14; widens RQ-CORE-021</t>
+        </is>
+      </c>
+      <c r="E287" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §14</t>
+        </is>
+      </c>
+      <c r="F287" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G287" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Excel import engine: template → upload → validate → error report → preview → maker → checker → approve → import → transa
+3. Expect the behaviour in blueprint §14; go-live: Core</t>
+        </is>
+      </c>
+      <c r="H287" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I287" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J287" s="2" t="inlineStr">
+        <is>
+          <t>core/bulk/engine.ts + /bulk/{importer}/template|preview|jobs/{id}/report|commit; the uploader commits their own job (no checker step).</t>
+        </is>
+      </c>
+      <c r="K287" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-112</t>
+        </is>
+      </c>
+      <c r="B288" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C288" s="2" t="inlineStr">
+        <is>
+          <t>Every import has an Import Batch ID and supports rollback/reversal of the complete batch (mandatory for salary, employee, attendance)</t>
+        </is>
+      </c>
+      <c r="D288" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §14; widens RQ-CORE-021</t>
+        </is>
+      </c>
+      <c r="E288" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §14</t>
+        </is>
+      </c>
+      <c r="F288" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G288" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Every import has an Import Batch ID and supports rollback/reversal of the complete batch (mandatory for salary, employee
+3. Expect the behaviour in blueprint §14; go-live: Core</t>
+        </is>
+      </c>
+      <c r="H288" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I288" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J288" s="2" t="inlineStr">
+        <is>
+          <t>core.bulk_jobs.id is the batch ID; savepoint rollback only on commit failure; no post-commit reversal.</t>
+        </is>
+      </c>
+      <c r="K288" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-120</t>
+        </is>
+      </c>
+      <c r="B289" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C289" s="2" t="inlineStr">
+        <is>
+          <t>Exit workflow: resignation → manager → Business Head → HR → notice → clearance → attendance freeze → leave encashment → salary/LOP → bonus/gratuity → recovery → asset clearance → F&amp;F → finance approval → payment → relieving/experience letter → exit</t>
+        </is>
+      </c>
+      <c r="D289" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §15; widens RQ-SEP-002, RQ-SEP-005</t>
+        </is>
+      </c>
+      <c r="E289" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §15</t>
+        </is>
+      </c>
+      <c r="F289" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G289" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Exit workflow: resignation → manager → Business Head → HR → notice → clearance → attendance freeze → leave encashment → 
+3. Expect the behaviour in blueprint §15; go-live: Core</t>
+        </is>
+      </c>
+      <c r="H289" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="I289" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J289" s="2" t="inlineStr">
+        <is>
+          <t>lifecycle/separation (chain, ceo-review), clearances, compute-fnf, pay (row lock, E2E-022), letters; no Business Head or Finance approval step in the seeded chain.</t>
+        </is>
+      </c>
+      <c r="K289" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-121</t>
+        </is>
+      </c>
+      <c r="B290" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C290" s="2" t="inlineStr">
+        <is>
+          <t>Separation types: resignation, termination, retirement, absconding, death, contract expiry, misconduct, restructuring, mutual separation</t>
+        </is>
+      </c>
+      <c r="D290" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §15; widens RQ-SEP-003</t>
+        </is>
+      </c>
+      <c r="E290" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §15</t>
+        </is>
+      </c>
+      <c r="F290" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G290" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Separation types: resignation, termination, retirement, absconding, death, contract expiry, misconduct, restructuring, m
+3. Expect the behaviour in blueprint §15; go-live: Core</t>
+        </is>
+      </c>
+      <c r="H290" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I290" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J290" s="2" t="inlineStr">
+        <is>
+          <t>core.separations initiated_by employee|hr, absconding path; no separation-type enum (death/retirement change gratuity eligibility and F&amp;F payee).</t>
+        </is>
+      </c>
+      <c r="K290" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-140</t>
+        </is>
+      </c>
+      <c r="B291" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C291" s="2" t="inlineStr">
+        <is>
+          <t>Performance: goals/KRA/KPI, weightage, mid-year, continuous feedback, self/manager appraisal, calibration, rating, increment/promotion linkage, 360, PIP</t>
+        </is>
+      </c>
+      <c r="D291" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §17</t>
+        </is>
+      </c>
+      <c r="E291" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §17</t>
+        </is>
+      </c>
+      <c r="F291" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G291" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Performance: goals/KRA/KPI, weightage, mid-year, continuous feedback, self/manager appraisal, calibration, rating, incre
+3. Expect the behaviour in blueprint §17; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H291" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I291" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J291" s="2" t="inlineStr">
+        <is>
+          <t>Only the probation review form.</t>
+        </is>
+      </c>
+      <c r="K291" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-141</t>
+        </is>
+      </c>
+      <c r="B292" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C292" s="2" t="inlineStr">
+        <is>
+          <t>OKR hierarchy Company → Business → Department → Individual objective</t>
+        </is>
+      </c>
+      <c r="D292" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §17</t>
+        </is>
+      </c>
+      <c r="E292" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §17</t>
+        </is>
+      </c>
+      <c r="F292" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G292" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: OKR hierarchy Company → Business → Department → Individual objective
+3. Expect the behaviour in blueprint §17; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H292" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I292" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J292" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="K292" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-150</t>
+        </is>
+      </c>
+      <c r="B293" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C293" s="2" t="inlineStr">
+        <is>
+          <t>Training lifecycle TNA → annual plan → nomination → training → attendance → assessment → feedback → effectiveness → record</t>
+        </is>
+      </c>
+      <c r="D293" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §18</t>
+        </is>
+      </c>
+      <c r="E293" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §18</t>
+        </is>
+      </c>
+      <c r="F293" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G293" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Training lifecycle TNA → annual plan → nomination → training → attendance → assessment → feedback → effectiveness → reco
+3. Expect the behaviour in blueprint §18; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H293" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I293" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J293" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="K293" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-151</t>
+        </is>
+      </c>
+      <c r="B294" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C294" s="2" t="inlineStr">
+        <is>
+          <t>Programme types: induction, technical, behavioural, compliance, safety, ISO, POSH, fire, LOTO, HIRA, SOP, leadership</t>
+        </is>
+      </c>
+      <c r="D294" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §18</t>
+        </is>
+      </c>
+      <c r="E294" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §18</t>
+        </is>
+      </c>
+      <c r="F294" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G294" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Programme types: induction, technical, behavioural, compliance, safety, ISO, POSH, fire, LOTO, HIRA, SOP, leadership
+3. Expect the behaviour in blueprint §18; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H294" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I294" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J294" s="2" t="inlineStr">
+        <is>
+          <t>None (hr_induction is a single onboarding task).</t>
+        </is>
+      </c>
+      <c r="K294" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-152</t>
+        </is>
+      </c>
+      <c r="B295" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C295" s="2" t="inlineStr">
+        <is>
+          <t>Skill matrix employee → process → skill → required/current level → gap → training, rating 0–5</t>
+        </is>
+      </c>
+      <c r="D295" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §18/§31</t>
+        </is>
+      </c>
+      <c r="E295" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §18/§31</t>
+        </is>
+      </c>
+      <c r="F295" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G295" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Skill matrix employee → process → skill → required/current level → gap → training, rating 0–5
+3. Expect the behaviour in blueprint §18/§31; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H295" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I295" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J295" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="K295" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-160</t>
+        </is>
+      </c>
+      <c r="B296" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C296" s="2" t="inlineStr">
+        <is>
+          <t>Critical-position identification, successor mapping, readiness, potential, risk, development plan</t>
+        </is>
+      </c>
+      <c r="D296" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §19</t>
+        </is>
+      </c>
+      <c r="E296" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §19</t>
+        </is>
+      </c>
+      <c r="F296" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G296" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Critical-position identification, successor mapping, readiness, potential, risk, development plan
+3. Expect the behaviour in blueprint §19; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H296" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I296" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J296" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="K296" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-161</t>
+        </is>
+      </c>
+      <c r="B297" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C297" s="2" t="inlineStr">
+        <is>
+          <t>9-box performance/potential framework and talent review</t>
+        </is>
+      </c>
+      <c r="D297" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §19</t>
+        </is>
+      </c>
+      <c r="E297" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §19</t>
+        </is>
+      </c>
+      <c r="F297" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G297" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: 9-box performance/potential framework and talent review
+3. Expect the behaviour in blueprint §19; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H297" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I297" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J297" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="K297" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-181</t>
+        </is>
+      </c>
+      <c r="B298" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C298" s="2" t="inlineStr">
+        <is>
+          <t>Confidential grievance and POSH case management with restricted access, evidence, investigation, IC actions, closure</t>
+        </is>
+      </c>
+      <c r="D298" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §22</t>
+        </is>
+      </c>
+      <c r="E298" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §22</t>
+        </is>
+      </c>
+      <c r="F298" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G298" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Confidential grievance and POSH case management with restricted access, evidence, investigation, IC actions, closure
+3. Expect the behaviour in blueprint §22; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H298" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I298" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J298" s="2" t="inlineStr">
+        <is>
+          <t>Schema only (ird.posh_cases, ird.grievances, ird.ic_members, posh_case_access_log); no API or UI.</t>
+        </is>
+      </c>
+      <c r="K298" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-192</t>
+        </is>
+      </c>
+      <c r="B299" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C299" s="2" t="inlineStr">
+        <is>
+          <t>Rewards: Star of Month/Quarter, Employee of Year, Safety, Innovation, Long Service, Spot awards with nomination/approval</t>
+        </is>
+      </c>
+      <c r="D299" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §23</t>
+        </is>
+      </c>
+      <c r="E299" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §23</t>
+        </is>
+      </c>
+      <c r="F299" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G299" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Rewards: Star of Month/Quarter, Employee of Year, Safety, Innovation, Long Service, Spot awards with nomination/approval
+3. Expect the behaviour in blueprint §23; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H299" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I299" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J299" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="K299" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-201</t>
+        </is>
+      </c>
+      <c r="B300" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C300" s="2" t="inlineStr">
+        <is>
+          <t>Document version control, expiry/renewal alerts, verification, e-sign, access control, download restrictions, audit</t>
+        </is>
+      </c>
+      <c r="D300" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §24</t>
+        </is>
+      </c>
+      <c r="E300" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §24</t>
+        </is>
+      </c>
+      <c r="F300" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G300" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Document version control, expiry/renewal alerts, verification, e-sign, access control, download restrictions, audit
+3. Expect the behaviour in blueprint §24; go-live: Core</t>
+        </is>
+      </c>
+      <c r="H300" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="I300" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J300" s="2" t="inlineStr">
+        <is>
+          <t>core.documents.expires_on/status columns; cmp.registrations expiry for licences; no versioning, verify flow or e-sign.</t>
+        </is>
+      </c>
+      <c r="K300" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-213</t>
+        </is>
+      </c>
+      <c r="B301" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C301" s="2" t="inlineStr">
+        <is>
+          <t>Training analytics: plan vs actual, hours, cost, effectiveness, skill gaps</t>
+        </is>
+      </c>
+      <c r="D301" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §25</t>
+        </is>
+      </c>
+      <c r="E301" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §25</t>
+        </is>
+      </c>
+      <c r="F301" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G301" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Training analytics: plan vs actual, hours, cost, effectiveness, skill gaps
+3. Expect the behaviour in blueprint §25; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H301" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I301" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J301" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="K301" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-220</t>
+        </is>
+      </c>
+      <c r="B302" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C302" s="2" t="inlineStr">
+        <is>
+          <t>Internal AI assistant (HR queries, policy search, requests, reports, exception analysis)</t>
+        </is>
+      </c>
+      <c r="D302" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §26</t>
+        </is>
+      </c>
+      <c r="E302" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §26</t>
+        </is>
+      </c>
+      <c r="F302" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G302" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Internal AI assistant (HR queries, policy search, requests, reports, exception analysis)
+3. Expect the behaviour in blueprint §26; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H302" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I302" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J302" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="K302" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-221</t>
+        </is>
+      </c>
+      <c r="B303" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C303" s="2" t="inlineStr">
+        <is>
+          <t>AI recruitment (resume parsing, JD match, ranking, duplicates, interview questions, rediscovery)</t>
+        </is>
+      </c>
+      <c r="D303" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §26</t>
+        </is>
+      </c>
+      <c r="E303" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §26</t>
+        </is>
+      </c>
+      <c r="F303" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G303" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: AI recruitment (resume parsing, JD match, ranking, duplicates, interview questions, rediscovery)
+3. Expect the behaviour in blueprint §26; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H303" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I303" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J303" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="K303" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-222</t>
+        </is>
+      </c>
+      <c r="B304" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C304" s="2" t="inlineStr">
+        <is>
+          <t>Predictive analytics (attrition risk, absenteeism, retirement, skill gaps, hiring, critical-position risk), advisory only</t>
+        </is>
+      </c>
+      <c r="D304" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §26</t>
+        </is>
+      </c>
+      <c r="E304" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §26</t>
+        </is>
+      </c>
+      <c r="F304" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G304" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Predictive analytics (attrition risk, absenteeism, retirement, skill gaps, hiring, critical-position risk), advisory onl
+3. Expect the behaviour in blueprint §26; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H304" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I304" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J304" s="2" t="inlineStr">
+        <is>
+          <t>Burnout index KPI only (RQ-RPT-116).</t>
+        </is>
+      </c>
+      <c r="K304" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-230</t>
+        </is>
+      </c>
+      <c r="B305" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C305" s="2" t="inlineStr">
+        <is>
+          <t>Approvals: sequential, parallel, conditional, amount-, grade-, plant- and department-based</t>
+        </is>
+      </c>
+      <c r="D305" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §27; widens RQ-WF-001, RQ-WF-011</t>
+        </is>
+      </c>
+      <c r="E305" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §27</t>
+        </is>
+      </c>
+      <c r="F305" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G305" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Approvals: sequential, parallel, conditional, amount-, grade-, plant- and department-based
+3. Expect the behaviour in blueprint §27; go-live: Core</t>
+        </is>
+      </c>
+      <c r="H305" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I305" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J305" s="2" t="inlineStr">
+        <is>
+          <t>workflow-definition.ts: sequential steps; approver = RM / FM / department_head / role / user; no parallel, condition or amount routing; plant-head step missing (RQ-WF-011).</t>
+        </is>
+      </c>
+      <c r="K305" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-240</t>
+        </is>
+      </c>
+      <c r="B306" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C306" s="2" t="inlineStr">
+        <is>
+          <t>RBAC: Super Admin, Group HR, Legal Entity HR, Plant HR, Department HR, Manager, Employee, Payroll, Finance, Auditor</t>
+        </is>
+      </c>
+      <c r="D306" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §28; widens RQ-RBAC-001, RQ-RBAC-008</t>
+        </is>
+      </c>
+      <c r="E306" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §28</t>
+        </is>
+      </c>
+      <c r="F306" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G306" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: RBAC: Super Admin, Group HR, Legal Entity HR, Plant HR, Department HR, Manager, Employee, Payroll, Finance, Auditor
+3. Expect the behaviour in blueprint §28; go-live: Core</t>
+        </is>
+      </c>
+      <c r="H306" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I306" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J306" s="2" t="inlineStr">
+        <is>
+          <t>Roles: employee, manager, hod, hr_ops, hr_head, payroll_admin, plant_head, ceo_cell, it_admin, super_admin; entity/plant HR via hr_ops scope; no Finance or read-only Auditor role.</t>
+        </is>
+      </c>
+      <c r="K306" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-241</t>
+        </is>
+      </c>
+      <c r="B307" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C307" s="2" t="inlineStr">
+        <is>
+          <t>Security: encryption, MFA, SSO, audit logs, session control, password policy, IP/device controls, backups, DR, data masking</t>
+        </is>
+      </c>
+      <c r="D307" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §28; widens RQ-NFR-004, RQ-NFR-009</t>
+        </is>
+      </c>
+      <c r="E307" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §28</t>
+        </is>
+      </c>
+      <c r="F307" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G307" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Security: encryption, MFA, SSO, audit logs, session control, password policy, IP/device controls, backups, DR, data mask
+3. Expect the behaviour in blueprint §28; go-live: Core</t>
+        </is>
+      </c>
+      <c r="H307" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="I307" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J307" s="2" t="inlineStr">
+        <is>
+          <t>Audit hash chain, sessions page, password history, backup/restore scripts, masking; sec.mfa_enrolments table but no MFA API/UI; no SSO, no IP allow-list (except Kent webhook); PII encryption is a plan (PII_ENCRYPTION_PLAN.md).</t>
+        </is>
+      </c>
+      <c r="K307" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-251</t>
+        </is>
+      </c>
+      <c r="B308" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C308" s="2" t="inlineStr">
+        <is>
+          <t>REST APIs, webhooks, SFTP, JSON/XML, OAuth 2.0</t>
+        </is>
+      </c>
+      <c r="D308" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §29</t>
+        </is>
+      </c>
+      <c r="E308" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §29</t>
+        </is>
+      </c>
+      <c r="F308" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G308" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: REST APIs, webhooks, SFTP, JSON/XML, OAuth 2.0
+3. Expect the behaviour in blueprint §29; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H308" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I308" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J308" s="2" t="inlineStr">
+        <is>
+          <t>REST/OpenAPI (oRPC); inbound Kent webhook + CSV drop; no outbound webhooks or OAuth2 client credentials.</t>
+        </is>
+      </c>
+      <c r="K308" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-260</t>
+        </is>
+      </c>
+      <c r="B309" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C309" s="2" t="inlineStr">
+        <is>
+          <t>Recommended stack: React/Next + TS, Flutter mobile, Java/Spring or .NET backend, PostgreSQL, Redis, OpenSearch, AWS/Azure, object storage, Power BI</t>
+        </is>
+      </c>
+      <c r="D309" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §30</t>
+        </is>
+      </c>
+      <c r="E309" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §30</t>
+        </is>
+      </c>
+      <c r="F309" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G309" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Recommended stack: React/Next + TS, Flutter mobile, Java/Spring or .NET backend, PostgreSQL, Redis, OpenSearch, AWS/Azur
+3. Expect the behaviour in blueprint §30; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H309" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I309" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J309" s="2" t="inlineStr">
+        <is>
+          <t>React + TS, PostgreSQL 17 as recommended; backend is Node/TypeScript (not Java/.NET); local-disk storage; no Redis/OpenSearch; mobile plan is PWA + Capacitor (MOBILE_RECOMMENDATION.md), not Flutter. Deviation needs an owner decision, not a rewrite.</t>
+        </is>
+      </c>
+      <c r="K309" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-271</t>
+        </is>
+      </c>
+      <c r="B310" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C310" s="2" t="inlineStr">
+        <is>
+          <t>Contractor manpower and labour compliance (CLRA: agency, licence, wage register, compliance)</t>
+        </is>
+      </c>
+      <c r="D310" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §31</t>
+        </is>
+      </c>
+      <c r="E310" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §31</t>
+        </is>
+      </c>
+      <c r="F310" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G310" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Contractor manpower and labour compliance (CLRA: agency, licence, wage register, compliance)
+3. Expect the behaviour in blueprint §31; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H310" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I310" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J310" s="2" t="inlineStr">
+        <is>
+          <t>Only category=contract; no contractor/agency master or contract-labour registers.</t>
+        </is>
+      </c>
+      <c r="K310" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-273</t>
+        </is>
+      </c>
+      <c r="B311" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C311" s="2" t="inlineStr">
+        <is>
+          <t>Medical fitness, PPE, safety training, certification expiry</t>
+        </is>
+      </c>
+      <c r="D311" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §31</t>
+        </is>
+      </c>
+      <c r="E311" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §31</t>
+        </is>
+      </c>
+      <c r="F311" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G311" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Medical fitness, PPE, safety training, certification expiry
+3. Expect the behaviour in blueprint §31; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H311" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I311" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J311" s="2" t="inlineStr">
+        <is>
+          <t>doc.types medical_fitness (blue_collar) without upload; PPE only as an asset category; no safety-training or certificate-expiry records.</t>
+        </is>
+      </c>
+      <c r="K311" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-281</t>
+        </is>
+      </c>
+      <c r="B312" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C312" s="2" t="inlineStr">
+        <is>
+          <t>Weekly vacancy, HR-pending and contractor-compliance reports</t>
+        </is>
+      </c>
+      <c r="D312" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §32</t>
+        </is>
+      </c>
+      <c r="E312" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §32</t>
+        </is>
+      </c>
+      <c r="F312" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G312" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Weekly vacancy, HR-pending and contractor-compliance reports
+3. Expect the behaviour in blueprint §32; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H312" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I312" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J312" s="2" t="inlineStr">
+        <is>
+          <t>None scheduled.</t>
+        </is>
+      </c>
+      <c r="K312" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-291</t>
+        </is>
+      </c>
+      <c r="B313" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C313" s="2" t="inlineStr">
+        <is>
+          <t>No-code form builder and report builder</t>
+        </is>
+      </c>
+      <c r="D313" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §33</t>
+        </is>
+      </c>
+      <c r="E313" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §33</t>
+        </is>
+      </c>
+      <c r="F313" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G313" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: No-code form builder and report builder
+3. Expect the behaviour in blueprint §33; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H313" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I313" s="3" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="J313" s="2" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="K313" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="2" t="inlineStr">
+        <is>
+          <t>RQ-BP-300</t>
+        </is>
+      </c>
+      <c r="B314" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="C314" s="2" t="inlineStr">
+        <is>
+          <t>Core entity set (legal_entity … import_batch, API log)</t>
+        </is>
+      </c>
+      <c r="D314" s="2" t="inlineStr">
+        <is>
+          <t>owner-docs "Rashmi Group HRMS Enterprise HRMS Requirements &amp; Feature Blueprint" (docx); /workspace/STATE/BLUEPRINT_GAP.md §34</t>
+        </is>
+      </c>
+      <c r="E314" s="2" t="inlineStr">
+        <is>
+          <t>Blueprint §34</t>
+        </is>
+      </c>
+      <c r="F314" s="2" t="inlineStr">
+        <is>
+          <t>per blueprint</t>
+        </is>
+      </c>
+      <c r="G314" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as hr_head (or the owning role)
+2. Exercise: Core entity set (legal_entity … import_batch, API log)
+3. Expect the behaviour in blueprint §34; go-live: Later</t>
+        </is>
+      </c>
+      <c r="H314" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="I314" s="3" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J314" s="2" t="inlineStr">
+        <is>
+          <t>Present: companies, locations, plants, departments, designations, grades, cost_centers, employees, employee_family, documents, employee_history, transfers, employee_salaries, salary_components, attendance (att.*), shifts, rosters, leave (lv.*), overtime, payroll runs/items/lines, arrears, fnf, onboarding, candidates, claims, travel, assets, compliance (cmp.*), grievance (schema), helpdesk, surveys, workflow, notifications, audit_log, bulk_jobs. Missing: division, section, job_family, job_level, position, profit centre, employee_address, employee_nominee (scheme-wise), employee_bank, employee_statutory, employee_education/experience, requisition, interview, offer, training, skill, competency, performance, goal, OKR, contractor, disciplinary_case, reward, api_log.</t>
+        </is>
+      </c>
+      <c r="K314" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K259"/>
+  <autoFilter ref="A1:K314"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15299,7 +18540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -15807,151 +19048,195 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>JF Joining form RML/HR/02/01</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>171</v>
+        <v>10</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>258</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n"/>
-      <c r="B24" s="2" t="n"/>
-      <c r="C24" s="2" t="n"/>
-      <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>BP Enterprise blueprint additions</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>33</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>Not software</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>196</v>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>313</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>P0</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="D26" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="E26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" s="2" t="n">
-        <v>100</v>
-      </c>
+      <c r="A26" s="2" t="n"/>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="C27" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="D27" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="E27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" s="2" t="n">
-        <v>96</v>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Not software</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P0</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>35</v>
+        <v>69</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>54</v>
+        <v>106</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>3</v>
+        <v>82</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>8</v>
+        <v>117</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>